<commit_message>
Chemistry: collapse water into two classes — potable vs non-potable
Muhannad: water should be two classifications. Merge tap (مياه الحنفية) + filter
(مياه فلتر) + bottled (مياه شرب/معبأة) into one potable «مياه صالحة للشرب»; keep
«مياه غير صالحة للشرب» (basin/standing/mobile) as non-potable. The merge runs
last in classify() so it also collapses water values from the per-sample_id
corrections. Supersedes the ubot→tap override (bottled no longer exists).

Result: مياه صالحة للشرب 1,050 · مياه غير صالحة للشرب 23. GSO bridge maps the
merged potable canonical → "Drinking Water". Regenerated parquets + clean/
chemistry sync + xlsx + dashboard (JS clean).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clean/chemistry/chem_heavy_metals_2024.xlsx
+++ b/clean/chemistry/chem_heavy_metals_2024.xlsx
@@ -3527,7 +3527,7 @@
       </c>
       <c r="CW11" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY11" t="inlineStr">
@@ -3790,7 +3790,7 @@
       </c>
       <c r="CW12" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY12" t="inlineStr">
@@ -4053,7 +4053,7 @@
       </c>
       <c r="CW13" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY13" t="inlineStr">
@@ -6976,7 +6976,7 @@
       </c>
       <c r="CW25" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY25" t="inlineStr">
@@ -7254,7 +7254,7 @@
       </c>
       <c r="CW26" t="inlineStr">
         <is>
-          <t>مياه شرب/معبأة</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY26" t="inlineStr">
@@ -7517,7 +7517,7 @@
       </c>
       <c r="CW27" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY27" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="CW28" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY28" t="inlineStr">
@@ -11948,7 +11948,7 @@
       </c>
       <c r="CW45" t="inlineStr">
         <is>
-          <t>مياه شرب/معبأة</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY45" t="inlineStr">
@@ -12211,7 +12211,7 @@
       </c>
       <c r="CW46" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY46" t="inlineStr">
@@ -14393,7 +14393,7 @@
       </c>
       <c r="CW55" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY55" t="inlineStr">
@@ -16619,7 +16619,7 @@
       </c>
       <c r="CW64" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY64" t="inlineStr">
@@ -16882,7 +16882,7 @@
       </c>
       <c r="CW65" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY65" t="inlineStr">
@@ -17145,7 +17145,7 @@
       </c>
       <c r="CW66" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY66" t="inlineStr">
@@ -17408,7 +17408,7 @@
       </c>
       <c r="CW67" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY67" t="inlineStr">
@@ -17671,7 +17671,7 @@
       </c>
       <c r="CW68" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY68" t="inlineStr">
@@ -17934,7 +17934,7 @@
       </c>
       <c r="CW69" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY69" t="inlineStr">
@@ -18197,7 +18197,7 @@
       </c>
       <c r="CW70" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY70" t="inlineStr">
@@ -18460,7 +18460,7 @@
       </c>
       <c r="CW71" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY71" t="inlineStr">
@@ -18723,7 +18723,7 @@
       </c>
       <c r="CW72" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY72" t="inlineStr">
@@ -18986,7 +18986,7 @@
       </c>
       <c r="CW73" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY73" t="inlineStr">
@@ -19225,7 +19225,7 @@
       </c>
       <c r="CW74" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY74" t="inlineStr">
@@ -19464,7 +19464,7 @@
       </c>
       <c r="CW75" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY75" t="inlineStr">
@@ -19703,7 +19703,7 @@
       </c>
       <c r="CW76" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY76" t="inlineStr">
@@ -19942,7 +19942,7 @@
       </c>
       <c r="CW77" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY77" t="inlineStr">
@@ -20181,7 +20181,7 @@
       </c>
       <c r="CW78" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY78" t="inlineStr">
@@ -20420,7 +20420,7 @@
       </c>
       <c r="CW79" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY79" t="inlineStr">
@@ -20659,7 +20659,7 @@
       </c>
       <c r="CW80" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY80" t="inlineStr">
@@ -20898,7 +20898,7 @@
       </c>
       <c r="CW81" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY81" t="inlineStr">
@@ -21137,7 +21137,7 @@
       </c>
       <c r="CW82" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY82" t="inlineStr">
@@ -21376,7 +21376,7 @@
       </c>
       <c r="CW83" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY83" t="inlineStr">
@@ -21615,7 +21615,7 @@
       </c>
       <c r="CW84" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY84" t="inlineStr">
@@ -21854,7 +21854,7 @@
       </c>
       <c r="CW85" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY85" t="inlineStr">
@@ -22096,7 +22096,7 @@
       </c>
       <c r="CW86" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY86" t="inlineStr">
@@ -22335,7 +22335,7 @@
       </c>
       <c r="CW87" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY87" t="inlineStr">
@@ -22574,7 +22574,7 @@
       </c>
       <c r="CW88" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY88" t="inlineStr">
@@ -22813,7 +22813,7 @@
       </c>
       <c r="CW89" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY89" t="inlineStr">
@@ -23052,7 +23052,7 @@
       </c>
       <c r="CW90" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY90" t="inlineStr">
@@ -23291,7 +23291,7 @@
       </c>
       <c r="CW91" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY91" t="inlineStr">
@@ -23530,7 +23530,7 @@
       </c>
       <c r="CW92" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY92" t="inlineStr">
@@ -23769,7 +23769,7 @@
       </c>
       <c r="CW93" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY93" t="inlineStr">
@@ -24011,7 +24011,7 @@
       </c>
       <c r="CW94" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY94" t="inlineStr">
@@ -24255,7 +24255,7 @@
       </c>
       <c r="CW95" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY95" t="inlineStr">
@@ -24497,7 +24497,7 @@
       </c>
       <c r="CW96" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY96" t="inlineStr">
@@ -24739,7 +24739,7 @@
       </c>
       <c r="CW97" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY97" t="inlineStr">
@@ -24981,7 +24981,7 @@
       </c>
       <c r="CW98" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY98" t="inlineStr">
@@ -25223,7 +25223,7 @@
       </c>
       <c r="CW99" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY99" t="inlineStr">
@@ -25465,7 +25465,7 @@
       </c>
       <c r="CW100" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY100" t="inlineStr">
@@ -25710,7 +25710,7 @@
       </c>
       <c r="CW101" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY101" t="inlineStr">
@@ -25952,7 +25952,7 @@
       </c>
       <c r="CW102" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY102" t="inlineStr">
@@ -26194,7 +26194,7 @@
       </c>
       <c r="CW103" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY103" t="inlineStr">
@@ -26436,7 +26436,7 @@
       </c>
       <c r="CW104" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY104" t="inlineStr">
@@ -26681,7 +26681,7 @@
       </c>
       <c r="CW105" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY105" t="inlineStr">
@@ -26926,7 +26926,7 @@
       </c>
       <c r="CW106" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY106" t="inlineStr">
@@ -27171,7 +27171,7 @@
       </c>
       <c r="CW107" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY107" t="inlineStr">
@@ -27416,7 +27416,7 @@
       </c>
       <c r="CW108" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY108" t="inlineStr">
@@ -27661,7 +27661,7 @@
       </c>
       <c r="CW109" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY109" t="inlineStr">
@@ -27909,7 +27909,7 @@
       </c>
       <c r="CW110" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY110" t="inlineStr">
@@ -28157,7 +28157,7 @@
       </c>
       <c r="CW111" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY111" t="inlineStr">
@@ -28405,7 +28405,7 @@
       </c>
       <c r="CW112" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY112" t="inlineStr">
@@ -29814,7 +29814,7 @@
       </c>
       <c r="CW118" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY118" t="inlineStr">
@@ -30056,7 +30056,7 @@
       </c>
       <c r="CW119" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY119" t="inlineStr">
@@ -30301,7 +30301,7 @@
       </c>
       <c r="CW120" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY120" t="inlineStr">
@@ -30543,7 +30543,7 @@
       </c>
       <c r="CW121" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY121" t="inlineStr">
@@ -30794,7 +30794,7 @@
       </c>
       <c r="CW122" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY122" t="inlineStr">
@@ -31045,7 +31045,7 @@
       </c>
       <c r="CW123" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY123" t="inlineStr">
@@ -31296,7 +31296,7 @@
       </c>
       <c r="CW124" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY124" t="inlineStr">
@@ -31547,7 +31547,7 @@
       </c>
       <c r="CW125" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY125" t="inlineStr">
@@ -31798,7 +31798,7 @@
       </c>
       <c r="CW126" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY126" t="inlineStr">
@@ -32049,7 +32049,7 @@
       </c>
       <c r="CW127" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY127" t="inlineStr">
@@ -32297,7 +32297,7 @@
       </c>
       <c r="CW128" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY128" t="inlineStr">
@@ -32545,7 +32545,7 @@
       </c>
       <c r="CW129" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY129" t="inlineStr">
@@ -32793,7 +32793,7 @@
       </c>
       <c r="CW130" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY130" t="inlineStr">
@@ -33041,7 +33041,7 @@
       </c>
       <c r="CW131" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY131" t="inlineStr">
@@ -33289,7 +33289,7 @@
       </c>
       <c r="CW132" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY132" t="inlineStr">
@@ -33537,7 +33537,7 @@
       </c>
       <c r="CW133" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY133" t="inlineStr">
@@ -33785,7 +33785,7 @@
       </c>
       <c r="CW134" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY134" t="inlineStr">
@@ -34033,7 +34033,7 @@
       </c>
       <c r="CW135" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY135" t="inlineStr">
@@ -34281,7 +34281,7 @@
       </c>
       <c r="CW136" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY136" t="inlineStr">
@@ -34529,7 +34529,7 @@
       </c>
       <c r="CW137" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY137" t="inlineStr">
@@ -34777,7 +34777,7 @@
       </c>
       <c r="CW138" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY138" t="inlineStr">
@@ -35025,7 +35025,7 @@
       </c>
       <c r="CW139" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY139" t="inlineStr">
@@ -35273,7 +35273,7 @@
       </c>
       <c r="CW140" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY140" t="inlineStr">
@@ -35521,7 +35521,7 @@
       </c>
       <c r="CW141" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY141" t="inlineStr">
@@ -35769,7 +35769,7 @@
       </c>
       <c r="CW142" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY142" t="inlineStr">
@@ -36017,7 +36017,7 @@
       </c>
       <c r="CW143" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY143" t="inlineStr">
@@ -36265,7 +36265,7 @@
       </c>
       <c r="CW144" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY144" t="inlineStr">
@@ -36513,7 +36513,7 @@
       </c>
       <c r="CW145" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY145" t="inlineStr">
@@ -36761,7 +36761,7 @@
       </c>
       <c r="CW146" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY146" t="inlineStr">
@@ -37009,7 +37009,7 @@
       </c>
       <c r="CW147" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY147" t="inlineStr">
@@ -37257,7 +37257,7 @@
       </c>
       <c r="CW148" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY148" t="inlineStr">
@@ -37514,7 +37514,7 @@
       </c>
       <c r="CW149" t="inlineStr">
         <is>
-          <t>مياه شرب/معبأة</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY149" t="inlineStr">
@@ -37771,7 +37771,7 @@
       </c>
       <c r="CW150" t="inlineStr">
         <is>
-          <t>مياه شرب/معبأة</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY150" t="inlineStr">
@@ -38019,7 +38019,7 @@
       </c>
       <c r="CW151" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY151" t="inlineStr">
@@ -38267,7 +38267,7 @@
       </c>
       <c r="CW152" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY152" t="inlineStr">
@@ -38515,7 +38515,7 @@
       </c>
       <c r="CW153" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY153" t="inlineStr">
@@ -38763,7 +38763,7 @@
       </c>
       <c r="CW154" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY154" t="inlineStr">
@@ -39011,7 +39011,7 @@
       </c>
       <c r="CW155" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY155" t="inlineStr">
@@ -39259,7 +39259,7 @@
       </c>
       <c r="CW156" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY156" t="inlineStr">
@@ -39507,7 +39507,7 @@
       </c>
       <c r="CW157" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY157" t="inlineStr">
@@ -39758,7 +39758,7 @@
       </c>
       <c r="CW158" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY158" t="inlineStr">
@@ -40009,7 +40009,7 @@
       </c>
       <c r="CW159" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY159" t="inlineStr">
@@ -40260,7 +40260,7 @@
       </c>
       <c r="CW160" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY160" t="inlineStr">
@@ -40511,7 +40511,7 @@
       </c>
       <c r="CW161" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY161" t="inlineStr">
@@ -40762,7 +40762,7 @@
       </c>
       <c r="CW162" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY162" t="inlineStr">
@@ -41013,7 +41013,7 @@
       </c>
       <c r="CW163" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY163" t="inlineStr">
@@ -41264,7 +41264,7 @@
       </c>
       <c r="CW164" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY164" t="inlineStr">
@@ -41515,7 +41515,7 @@
       </c>
       <c r="CW165" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY165" t="inlineStr">
@@ -41775,7 +41775,7 @@
       </c>
       <c r="CW166" t="inlineStr">
         <is>
-          <t>مياه شرب/معبأة</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY166" t="inlineStr">
@@ -42026,7 +42026,7 @@
       </c>
       <c r="CW167" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY167" t="inlineStr">
@@ -42277,7 +42277,7 @@
       </c>
       <c r="CW168" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY168" t="inlineStr">
@@ -42528,7 +42528,7 @@
       </c>
       <c r="CW169" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY169" t="inlineStr">
@@ -42779,7 +42779,7 @@
       </c>
       <c r="CW170" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY170" t="inlineStr">
@@ -43030,7 +43030,7 @@
       </c>
       <c r="CW171" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY171" t="inlineStr">
@@ -43281,7 +43281,7 @@
       </c>
       <c r="CW172" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY172" t="inlineStr">
@@ -43532,7 +43532,7 @@
       </c>
       <c r="CW173" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY173" t="inlineStr">
@@ -43783,7 +43783,7 @@
       </c>
       <c r="CW174" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY174" t="inlineStr">
@@ -44034,7 +44034,7 @@
       </c>
       <c r="CW175" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY175" t="inlineStr">
@@ -44285,7 +44285,7 @@
       </c>
       <c r="CW176" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY176" t="inlineStr">
@@ -44536,7 +44536,7 @@
       </c>
       <c r="CW177" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY177" t="inlineStr">
@@ -44787,7 +44787,7 @@
       </c>
       <c r="CW178" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY178" t="inlineStr">
@@ -45038,7 +45038,7 @@
       </c>
       <c r="CW179" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY179" t="inlineStr">
@@ -45289,7 +45289,7 @@
       </c>
       <c r="CW180" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY180" t="inlineStr">
@@ -45540,7 +45540,7 @@
       </c>
       <c r="CW181" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY181" t="inlineStr">
@@ -45800,7 +45800,7 @@
       </c>
       <c r="CW182" t="inlineStr">
         <is>
-          <t>مياه شرب/معبأة</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY182" t="inlineStr">
@@ -46051,7 +46051,7 @@
       </c>
       <c r="CW183" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY183" t="inlineStr">
@@ -46302,7 +46302,7 @@
       </c>
       <c r="CW184" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY184" t="inlineStr">
@@ -46553,7 +46553,7 @@
       </c>
       <c r="CW185" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY185" t="inlineStr">
@@ -46804,7 +46804,7 @@
       </c>
       <c r="CW186" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY186" t="inlineStr">
@@ -47055,7 +47055,7 @@
       </c>
       <c r="CW187" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY187" t="inlineStr">
@@ -47306,7 +47306,7 @@
       </c>
       <c r="CW188" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY188" t="inlineStr">
@@ -47557,7 +47557,7 @@
       </c>
       <c r="CW189" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY189" t="inlineStr">
@@ -47808,7 +47808,7 @@
       </c>
       <c r="CW190" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY190" t="inlineStr">
@@ -48062,7 +48062,7 @@
       </c>
       <c r="CW191" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY191" t="inlineStr">
@@ -48316,7 +48316,7 @@
       </c>
       <c r="CW192" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY192" t="inlineStr">
@@ -48570,7 +48570,7 @@
       </c>
       <c r="CW193" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY193" t="inlineStr">
@@ -48824,7 +48824,7 @@
       </c>
       <c r="CW194" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY194" t="inlineStr">
@@ -49078,7 +49078,7 @@
       </c>
       <c r="CW195" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY195" t="inlineStr">
@@ -49332,7 +49332,7 @@
       </c>
       <c r="CW196" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY196" t="inlineStr">
@@ -49586,7 +49586,7 @@
       </c>
       <c r="CW197" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY197" t="inlineStr">
@@ -49840,7 +49840,7 @@
       </c>
       <c r="CW198" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY198" t="inlineStr">
@@ -50094,7 +50094,7 @@
       </c>
       <c r="CW199" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY199" t="inlineStr">
@@ -50348,7 +50348,7 @@
       </c>
       <c r="CW200" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY200" t="inlineStr">
@@ -50602,7 +50602,7 @@
       </c>
       <c r="CW201" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY201" t="inlineStr">
@@ -50856,7 +50856,7 @@
       </c>
       <c r="CW202" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY202" t="inlineStr">
@@ -51110,7 +51110,7 @@
       </c>
       <c r="CW203" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY203" t="inlineStr">
@@ -51364,7 +51364,7 @@
       </c>
       <c r="CW204" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY204" t="inlineStr">
@@ -51612,7 +51612,7 @@
       </c>
       <c r="CW205" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY205" t="inlineStr">
@@ -51863,7 +51863,7 @@
       </c>
       <c r="CW206" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY206" t="inlineStr">
@@ -52114,7 +52114,7 @@
       </c>
       <c r="CW207" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY207" t="inlineStr">
@@ -52370,7 +52370,7 @@
       </c>
       <c r="CW208" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY208" t="inlineStr">
@@ -52621,7 +52621,7 @@
       </c>
       <c r="CW209" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY209" t="inlineStr">
@@ -52872,7 +52872,7 @@
       </c>
       <c r="CW210" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY210" t="inlineStr">
@@ -53123,7 +53123,7 @@
       </c>
       <c r="CW211" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY211" t="inlineStr">
@@ -53374,7 +53374,7 @@
       </c>
       <c r="CW212" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY212" t="inlineStr">
@@ -54310,7 +54310,7 @@
       </c>
       <c r="CW216" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY216" t="inlineStr">
@@ -54565,7 +54565,7 @@
       </c>
       <c r="CW217" t="inlineStr">
         <is>
-          <t>مياه شرب/معبأة</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY217" t="inlineStr">
@@ -54811,7 +54811,7 @@
       </c>
       <c r="CW218" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY218" t="inlineStr">
@@ -55057,7 +55057,7 @@
       </c>
       <c r="CW219" t="inlineStr">
         <is>
-          <t>مياه فلتر</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY219" t="inlineStr">
@@ -55295,7 +55295,7 @@
       </c>
       <c r="CW220" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY220" t="inlineStr">
@@ -55533,7 +55533,7 @@
       </c>
       <c r="CW221" t="inlineStr">
         <is>
-          <t>مياه الحنفية</t>
+          <t>مياه صالحة للشرب</t>
         </is>
       </c>
       <c r="CY221" t="inlineStr">

</xml_diff>